<commit_message>
Updated process to include detailed statistics
</commit_message>
<xml_diff>
--- a/mtg_data.xlsx
+++ b/mtg_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VS Code\MTG Analysis\venv\project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7521C24-FE88-4BD4-9EFB-F611093DA03B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40825996-5942-4335-B49F-6B450D852FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1137F1D1-D151-4314-AE7F-A3B4E1F9669F}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="32">
   <si>
     <t>game_id</t>
   </si>
@@ -111,6 +111,30 @@
   </si>
   <si>
     <t>Bloomburrow</t>
+  </si>
+  <si>
+    <t>damage_dealt</t>
+  </si>
+  <si>
+    <t>damage_received</t>
+  </si>
+  <si>
+    <t>health_lost</t>
+  </si>
+  <si>
+    <t>health_gained</t>
+  </si>
+  <si>
+    <t>creature_killed</t>
+  </si>
+  <si>
+    <t>creature_lost</t>
+  </si>
+  <si>
+    <t>vip_kill</t>
+  </si>
+  <si>
+    <t>vip_loss</t>
   </si>
 </sst>
 </file>
@@ -146,10 +170,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -485,15 +512,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31210DC3-84DF-4463-A036-811DC51179A3}">
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:M59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.140625" customWidth="1"/>
-    <col min="11" max="11" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="13" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -509,12 +536,32 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -533,7 +580,7 @@
       <c r="H2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -552,7 +599,7 @@
       <c r="H3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -571,7 +618,7 @@
       <c r="H4" s="1"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -589,7 +636,7 @@
       </c>
       <c r="H5" s="1"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>2</v>
       </c>
@@ -607,7 +654,7 @@
       </c>
       <c r="H6" s="1"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>2</v>
       </c>
@@ -624,7 +671,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>2</v>
       </c>
@@ -641,7 +688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>3</v>
       </c>
@@ -658,7 +705,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>3</v>
       </c>
@@ -675,7 +722,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>3</v>
       </c>
@@ -692,7 +739,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>3</v>
       </c>
@@ -709,7 +756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>4</v>
       </c>
@@ -726,7 +773,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>4</v>
       </c>
@@ -743,7 +790,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>4</v>
       </c>
@@ -760,7 +807,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>4</v>
       </c>
@@ -1321,7 +1368,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>14</v>
       </c>
@@ -1338,7 +1385,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>14</v>
       </c>
@@ -1355,7 +1402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>14</v>
       </c>
@@ -1372,7 +1419,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>15</v>
       </c>
@@ -1388,8 +1435,32 @@
       <c r="E52" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F52">
+        <v>32</v>
+      </c>
+      <c r="G52">
+        <v>57</v>
+      </c>
+      <c r="H52" s="1">
+        <v>44</v>
+      </c>
+      <c r="I52" s="1">
+        <v>4</v>
+      </c>
+      <c r="J52" s="1">
+        <v>3</v>
+      </c>
+      <c r="K52" s="1">
+        <v>16</v>
+      </c>
+      <c r="L52" s="1">
+        <v>0</v>
+      </c>
+      <c r="M52" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>15</v>
       </c>
@@ -1405,8 +1476,32 @@
       <c r="E53" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F53">
+        <v>84</v>
+      </c>
+      <c r="G53">
+        <v>61</v>
+      </c>
+      <c r="H53" s="1">
+        <v>42</v>
+      </c>
+      <c r="I53" s="1">
+        <v>2</v>
+      </c>
+      <c r="J53" s="1">
+        <v>25</v>
+      </c>
+      <c r="K53" s="1">
+        <v>19</v>
+      </c>
+      <c r="L53" s="1">
+        <v>7</v>
+      </c>
+      <c r="M53" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>15</v>
       </c>
@@ -1422,8 +1517,32 @@
       <c r="E54" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F54">
+        <v>40</v>
+      </c>
+      <c r="G54">
+        <v>53</v>
+      </c>
+      <c r="H54" s="1">
+        <v>43</v>
+      </c>
+      <c r="I54" s="1">
+        <v>0</v>
+      </c>
+      <c r="J54" s="1">
+        <v>18</v>
+      </c>
+      <c r="K54" s="1">
+        <v>8</v>
+      </c>
+      <c r="L54" s="1">
+        <v>3</v>
+      </c>
+      <c r="M54" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>15</v>
       </c>
@@ -1439,9 +1558,197 @@
       <c r="E55" s="1">
         <v>1</v>
       </c>
+      <c r="F55">
+        <v>75</v>
+      </c>
+      <c r="G55">
+        <v>70</v>
+      </c>
+      <c r="H55" s="1">
+        <v>60</v>
+      </c>
+      <c r="I55" s="1">
+        <v>34</v>
+      </c>
+      <c r="J55" s="1">
+        <v>7</v>
+      </c>
+      <c r="K55" s="1">
+        <v>13</v>
+      </c>
+      <c r="L55" s="1">
+        <v>0</v>
+      </c>
+      <c r="M55" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>16</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E56" s="1">
+        <v>3</v>
+      </c>
+      <c r="F56">
+        <v>159</v>
+      </c>
+      <c r="G56">
+        <v>84</v>
+      </c>
+      <c r="H56" s="1">
+        <v>76</v>
+      </c>
+      <c r="I56" s="1">
+        <v>0</v>
+      </c>
+      <c r="J56" s="1">
+        <v>19</v>
+      </c>
+      <c r="K56" s="1">
+        <v>7</v>
+      </c>
+      <c r="L56" s="1">
+        <v>2</v>
+      </c>
+      <c r="M56" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>16</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E57" s="1">
+        <v>2</v>
+      </c>
+      <c r="F57">
+        <v>69</v>
+      </c>
+      <c r="G57">
+        <v>66</v>
+      </c>
+      <c r="H57" s="1">
+        <v>51</v>
+      </c>
+      <c r="I57" s="1">
+        <v>11</v>
+      </c>
+      <c r="J57" s="1">
+        <v>10</v>
+      </c>
+      <c r="K57" s="1">
+        <v>11</v>
+      </c>
+      <c r="L57" s="1">
+        <v>0</v>
+      </c>
+      <c r="M57" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>16</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E58" s="1">
+        <v>1</v>
+      </c>
+      <c r="F58">
+        <v>143</v>
+      </c>
+      <c r="G58">
+        <v>64</v>
+      </c>
+      <c r="H58" s="1">
+        <v>43</v>
+      </c>
+      <c r="I58" s="1">
+        <v>39</v>
+      </c>
+      <c r="J58" s="1">
+        <v>8</v>
+      </c>
+      <c r="K58" s="1">
+        <v>12</v>
+      </c>
+      <c r="L58" s="1">
+        <v>1</v>
+      </c>
+      <c r="M58" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>16</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E59" s="1">
+        <v>4</v>
+      </c>
+      <c r="F59">
+        <v>6</v>
+      </c>
+      <c r="G59">
+        <v>83</v>
+      </c>
+      <c r="H59" s="1">
+        <v>45</v>
+      </c>
+      <c r="I59" s="1">
+        <v>3</v>
+      </c>
+      <c r="J59" s="1">
+        <v>0</v>
+      </c>
+      <c r="K59" s="1">
+        <v>9</v>
+      </c>
+      <c r="L59" s="1">
+        <v>0</v>
+      </c>
+      <c r="M59" s="1">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E55" xr:uid="{31210DC3-84DF-4463-A036-811DC51179A3}"/>
+  <autoFilter ref="A1:M1" xr:uid="{31210DC3-84DF-4463-A036-811DC51179A3}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updating data with last match
</commit_message>
<xml_diff>
--- a/mtg_data.xlsx
+++ b/mtg_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VS Code\MTG Analysis\venv\project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE9B0606-8B29-447B-B1DA-1C842C49207F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBC2EC39-CE8C-4092-B242-E91938818219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1137F1D1-D151-4314-AE7F-A3B4E1F9669F}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$107</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="62">
   <si>
     <t>game_id</t>
   </si>
@@ -599,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31210DC3-84DF-4463-A036-811DC51179A3}">
-  <dimension ref="A1:G103"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="19.08984375" customWidth="1"/>
@@ -2977,8 +2977,100 @@
         <v>43</v>
       </c>
     </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A104" s="1">
+        <v>28</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E104" s="1">
+        <v>4</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G104" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A105" s="1">
+        <v>28</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E105" s="1">
+        <v>2</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G105" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A106" s="1">
+        <v>28</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E106" s="1">
+        <v>1</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G106" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A107" s="1">
+        <v>28</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E107" s="1">
+        <v>3</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G107" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G103" xr:uid="{31210DC3-84DF-4463-A036-811DC51179A3}"/>
+  <autoFilter ref="A1:G107" xr:uid="{31210DC3-84DF-4463-A036-811DC51179A3}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated with latest game data
</commit_message>
<xml_diff>
--- a/mtg_data.xlsx
+++ b/mtg_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VS Code\MTG Analysis\venv\project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBC2EC39-CE8C-4092-B242-E91938818219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49EDE69C-185E-42EB-A17F-9F89327E5161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1137F1D1-D151-4314-AE7F-A3B4E1F9669F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1137F1D1-D151-4314-AE7F-A3B4E1F9669F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="62">
   <si>
     <t>game_id</t>
   </si>
@@ -599,16 +599,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31210DC3-84DF-4463-A036-811DC51179A3}">
-  <dimension ref="A1:G107"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:G111"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="19.08984375" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
     <col min="4" max="4" width="21" customWidth="1"/>
-    <col min="6" max="6" width="14.90625" customWidth="1"/>
-    <col min="7" max="7" width="21.1796875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="14.85546875" customWidth="1"/>
+    <col min="7" max="7" width="21.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -631,7 +631,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -654,7 +654,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -677,7 +677,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -700,7 +700,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -723,7 +723,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>2</v>
       </c>
@@ -746,7 +746,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>2</v>
       </c>
@@ -769,7 +769,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>2</v>
       </c>
@@ -792,7 +792,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>3</v>
       </c>
@@ -815,7 +815,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>3</v>
       </c>
@@ -838,7 +838,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>3</v>
       </c>
@@ -861,7 +861,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>3</v>
       </c>
@@ -884,7 +884,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>4</v>
       </c>
@@ -907,7 +907,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>4</v>
       </c>
@@ -930,7 +930,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>4</v>
       </c>
@@ -953,7 +953,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>4</v>
       </c>
@@ -976,7 +976,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>5</v>
       </c>
@@ -999,7 +999,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>5</v>
       </c>
@@ -1022,7 +1022,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>5</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>5</v>
       </c>
@@ -1068,7 +1068,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>7</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>7</v>
       </c>
@@ -1114,7 +1114,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>7</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>7</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>8</v>
       </c>
@@ -1183,7 +1183,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>8</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>8</v>
       </c>
@@ -1229,7 +1229,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>8</v>
       </c>
@@ -1252,7 +1252,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>9</v>
       </c>
@@ -1275,7 +1275,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>9</v>
       </c>
@@ -1298,7 +1298,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>9</v>
       </c>
@@ -1321,7 +1321,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>10</v>
       </c>
@@ -1344,7 +1344,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>10</v>
       </c>
@@ -1367,7 +1367,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>10</v>
       </c>
@@ -1390,7 +1390,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>10</v>
       </c>
@@ -1413,7 +1413,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>11</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>11</v>
       </c>
@@ -1459,7 +1459,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>11</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>11</v>
       </c>
@@ -1505,7 +1505,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>12</v>
       </c>
@@ -1528,7 +1528,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>12</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>12</v>
       </c>
@@ -1574,7 +1574,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>12</v>
       </c>
@@ -1597,7 +1597,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>13</v>
       </c>
@@ -1620,7 +1620,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>13</v>
       </c>
@@ -1643,7 +1643,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>13</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>13</v>
       </c>
@@ -1689,7 +1689,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>14</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>14</v>
       </c>
@@ -1735,7 +1735,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>14</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>14</v>
       </c>
@@ -1781,7 +1781,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>15</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>15</v>
       </c>
@@ -1827,7 +1827,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>15</v>
       </c>
@@ -1850,7 +1850,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>15</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>16</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>16</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>16</v>
       </c>
@@ -1942,7 +1942,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>16</v>
       </c>
@@ -1965,7 +1965,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>17</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>17</v>
       </c>
@@ -2011,7 +2011,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>17</v>
       </c>
@@ -2034,7 +2034,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>17</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>18</v>
       </c>
@@ -2080,7 +2080,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>18</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>18</v>
       </c>
@@ -2126,7 +2126,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>18</v>
       </c>
@@ -2149,7 +2149,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>19</v>
       </c>
@@ -2172,7 +2172,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>19</v>
       </c>
@@ -2195,7 +2195,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>19</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>19</v>
       </c>
@@ -2241,7 +2241,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>20</v>
       </c>
@@ -2264,7 +2264,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>20</v>
       </c>
@@ -2287,7 +2287,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>20</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>20</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>21</v>
       </c>
@@ -2356,7 +2356,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>21</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>21</v>
       </c>
@@ -2402,7 +2402,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>21</v>
       </c>
@@ -2425,7 +2425,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>22</v>
       </c>
@@ -2448,7 +2448,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>22</v>
       </c>
@@ -2471,7 +2471,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>22</v>
       </c>
@@ -2494,7 +2494,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>22</v>
       </c>
@@ -2517,7 +2517,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>23</v>
       </c>
@@ -2540,7 +2540,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>23</v>
       </c>
@@ -2563,7 +2563,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>23</v>
       </c>
@@ -2586,7 +2586,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>23</v>
       </c>
@@ -2609,7 +2609,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>24</v>
       </c>
@@ -2632,7 +2632,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>24</v>
       </c>
@@ -2655,7 +2655,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>24</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>24</v>
       </c>
@@ -2701,7 +2701,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>25</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>25</v>
       </c>
@@ -2747,7 +2747,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>25</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>25</v>
       </c>
@@ -2793,7 +2793,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>26</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>26</v>
       </c>
@@ -2839,7 +2839,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>26</v>
       </c>
@@ -2862,7 +2862,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>26</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>27</v>
       </c>
@@ -2908,7 +2908,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>27</v>
       </c>
@@ -2931,7 +2931,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>27</v>
       </c>
@@ -2954,7 +2954,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>27</v>
       </c>
@@ -2977,7 +2977,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>28</v>
       </c>
@@ -3000,7 +3000,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>28</v>
       </c>
@@ -3023,7 +3023,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>28</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>28</v>
       </c>
@@ -3067,6 +3067,98 @@
       </c>
       <c r="G107" s="1" t="s">
         <v>46</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A108" s="1">
+        <v>29</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E108" s="1">
+        <v>4</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G108" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A109" s="1">
+        <v>29</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E109" s="1">
+        <v>3</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G109" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A110" s="1">
+        <v>29</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E110" s="1">
+        <v>1</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G110" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A111" s="1">
+        <v>29</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E111" s="1">
+        <v>2</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G111" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating with latest game data
</commit_message>
<xml_diff>
--- a/mtg_data.xlsx
+++ b/mtg_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VS Code\MTG Analysis\venv\project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49EDE69C-185E-42EB-A17F-9F89327E5161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A7CB08F-EFB9-41ED-AB7B-D7FE8B9D1042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1137F1D1-D151-4314-AE7F-A3B4E1F9669F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="69">
   <si>
     <t>game_id</t>
   </si>
@@ -225,6 +225,27 @@
   </si>
   <si>
     <t>Science!</t>
+  </si>
+  <si>
+    <t>Marvel</t>
+  </si>
+  <si>
+    <t>Wakanda Forever</t>
+  </si>
+  <si>
+    <t>Selesenya {G} {W}</t>
+  </si>
+  <si>
+    <t>Avengers Assemble</t>
+  </si>
+  <si>
+    <t>Doom Prevails</t>
+  </si>
+  <si>
+    <t>Fantastic Four</t>
+  </si>
+  <si>
+    <t>Ink-Tread {xBlacl}</t>
   </si>
 </sst>
 </file>
@@ -599,7 +620,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31210DC3-84DF-4463-A036-811DC51179A3}">
-  <dimension ref="A1:G111"/>
+  <dimension ref="A1:G115"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="19.140625" customWidth="1"/>
@@ -3161,6 +3182,98 @@
         <v>50</v>
       </c>
     </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A112" s="1">
+        <v>30</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E112" s="1">
+        <v>4</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G112" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A113" s="1">
+        <v>30</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E113" s="1">
+        <v>2</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G113" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A114" s="1">
+        <v>30</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E114" s="1">
+        <v>1</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A115" s="1">
+        <v>30</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E115" s="1">
+        <v>3</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G107" xr:uid="{31210DC3-84DF-4463-A036-811DC51179A3}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>